<commit_message>
Updated Zn and Cu plots
</commit_message>
<xml_diff>
--- a/Copper/5. Statistical data analysis/Multiple linear regression/MLR_flagged_obs.xlsx
+++ b/Copper/5. Statistical data analysis/Multiple linear regression/MLR_flagged_obs.xlsx
@@ -132,13 +132,13 @@
     <t xml:space="preserve">Main Stem</t>
   </si>
   <si>
-    <t xml:space="preserve">Non-Perennial Tribs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perennial Developed Tribs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perennial Tribs</t>
+    <t xml:space="preserve">NP Tribs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P Tribs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD Tribs</t>
   </si>
   <si>
     <t xml:space="preserve">BSL4.3</t>
@@ -1148,16 +1148,16 @@
         <v>40</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>0.037037037037037</v>
+        <v>0.259259259259259</v>
       </c>
       <c r="D4" t="n">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="E4" t="n">
-        <v>0.326424870466321</v>
+        <v>0.282383419689119</v>
       </c>
     </row>
     <row r="5">
@@ -1165,16 +1165,16 @@
         <v>41</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.259259259259259</v>
+        <v>0.037037037037037</v>
       </c>
       <c r="D5" t="n">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="E5" t="n">
-        <v>0.282383419689119</v>
+        <v>0.326424870466321</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Sensitivity analysis of humic acid content for Zn and Cu bioavailability
</commit_message>
<xml_diff>
--- a/Copper/5. Statistical data analysis/Multiple linear regression/MLR_flagged_obs.xlsx
+++ b/Copper/5. Statistical data analysis/Multiple linear regression/MLR_flagged_obs.xlsx
@@ -1120,10 +1120,10 @@
         <v>0.296296296296296</v>
       </c>
       <c r="D2" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="E2" t="n">
-        <v>0.341968911917098</v>
+        <v>0.329015544041451</v>
       </c>
     </row>
     <row r="3">
@@ -1131,16 +1131,16 @@
         <v>39</v>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.407407407407407</v>
+        <v>0.296296296296296</v>
       </c>
       <c r="D3" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0492227979274611</v>
+        <v>0.0362694300518135</v>
       </c>
     </row>
     <row r="4">
@@ -1148,16 +1148,16 @@
         <v>40</v>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>0.259259259259259</v>
+        <v>0.185185185185185</v>
       </c>
       <c r="D4" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="E4" t="n">
-        <v>0.282383419689119</v>
+        <v>0.253886010362694</v>
       </c>
     </row>
     <row r="5">
@@ -1171,32 +1171,30 @@
         <v>0.037037037037037</v>
       </c>
       <c r="D5" t="n">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="E5" t="n">
-        <v>0.326424870466321</v>
+        <v>0.303108808290155</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s">
-        <v>42</v>
-      </c>
+      <c r="A6"/>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.037037037037037</v>
+        <v>0.185185185185185</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0103626943005181</v>
+        <v>0.077720207253886</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B7" t="n">
         <v>1</v>
@@ -1205,15 +1203,15 @@
         <v>0.037037037037037</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>0.00259067357512953</v>
+        <v>0.0103626943005181</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B8" t="n">
         <v>1</v>
@@ -1222,15 +1220,15 @@
         <v>0.037037037037037</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0284974093264249</v>
+        <v>0.00259067357512953</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B9" t="n">
         <v>1</v>
@@ -1247,13 +1245,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>0.222222222222222</v>
+        <v>0.037037037037037</v>
       </c>
       <c r="D10" t="n">
         <v>11</v>
@@ -1264,13 +1262,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C11" t="n">
-        <v>0.037037037037037</v>
+        <v>0.222222222222222</v>
       </c>
       <c r="D11" t="n">
         <v>11</v>
@@ -1281,41 +1279,41 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>0.185185185185185</v>
+        <v>0.037037037037037</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0129533678756477</v>
+        <v>0.0284974093264249</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>0.037037037037037</v>
+        <v>0.185185185185185</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0103626943005181</v>
+        <v>0.0129533678756477</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B14" t="n">
         <v>1</v>
@@ -1324,72 +1322,72 @@
         <v>0.037037037037037</v>
       </c>
       <c r="D14" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0284974093264249</v>
+        <v>0.0103626943005181</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0740740740740741</v>
+        <v>0.037037037037037</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E15" t="n">
-        <v>0.00518134715025907</v>
+        <v>0.0284974093264249</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>0.037037037037037</v>
+        <v>0.0740740740740741</v>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0284974093264249</v>
+        <v>0.00518134715025907</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>0.111111111111111</v>
+        <v>0.037037037037037</v>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0155440414507772</v>
+        <v>0.0284974093264249</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>0.037037037037037</v>
+        <v>0.111111111111111</v>
       </c>
       <c r="D18" t="n">
         <v>6</v>
@@ -1400,7 +1398,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B19" t="n">
         <v>1</v>
@@ -1409,15 +1407,15 @@
         <v>0.037037037037037</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0129533678756477</v>
+        <v>0.0155440414507772</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B20" t="n">
         <v>1</v>
@@ -1426,32 +1424,32 @@
         <v>0.037037037037037</v>
       </c>
       <c r="D20" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0207253886010363</v>
+        <v>0.0129533678756477</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B21" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>0.259259259259259</v>
+        <v>0.037037037037037</v>
       </c>
       <c r="D21" t="n">
-        <v>131</v>
+        <v>8</v>
       </c>
       <c r="E21" t="n">
-        <v>0.339378238341969</v>
+        <v>0.0207253886010363</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B22" t="n">
         <v>7</v>
@@ -1460,26 +1458,43 @@
         <v>0.259259259259259</v>
       </c>
       <c r="D22" t="n">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="E22" t="n">
-        <v>0.284974093264249</v>
+        <v>0.339378238341969</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" t="n">
+        <v>7</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.259259259259259</v>
+      </c>
+      <c r="D23" t="n">
+        <v>110</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.284974093264249</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
         <v>59</v>
       </c>
-      <c r="B23" t="n">
+      <c r="B24" t="n">
         <v>13</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C24" t="n">
         <v>0.481481481481481</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>145</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E24" t="n">
         <v>0.375647668393782</v>
       </c>
     </row>

</xml_diff>